<commit_message>
update bm y fichero datos
</commit_message>
<xml_diff>
--- a/datos/2026-02-01-rendimientos-analisis-desviaciones.xlsx
+++ b/datos/2026-02-01-rendimientos-analisis-desviaciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/34bf2af71bbc2e43/Documentos/GitHub/master-queseria/website/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="921" documentId="8_{566A70F3-096B-4476-B336-90A9B7DB3344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADE933D9-5892-4042-848B-69915A688E4D}"/>
+  <xr:revisionPtr revIDLastSave="943" documentId="8_{566A70F3-096B-4476-B336-90A9B7DB3344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{031111F0-0B3B-4236-9EEB-9AEB9ED8259A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="675" activeTab="1" xr2:uid="{6977E7F1-D64B-47FE-B2A7-D4E9B0399E18}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="675" activeTab="2" xr2:uid="{6977E7F1-D64B-47FE-B2A7-D4E9B0399E18}"/>
   </bookViews>
   <sheets>
     <sheet name="Liquidación leche" sheetId="17" r:id="rId1"/>
@@ -957,7 +957,7 @@
     <definedName name="zzzzzzzzzzzzzzzzzz" localSheetId="5" hidden="1">{"QQQ",#N/A,FALSE,"RIEP"}</definedName>
     <definedName name="zzzzzzzzzzzzzzzzzz" hidden="1">{"QQQ",#N/A,FALSE,"RIEP"}</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2670,10 +2670,10 @@
                   <c:v>89.914599659044001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.6286777499999996</c:v>
+                  <c:v>5.3713874999999982</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>83.382041907905304</c:v>
+                  <c:v>83.440017977571969</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2739,10 +2739,10 @@
                   <c:v>4.2403446035919998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.5022883777777785</c:v>
+                  <c:v>3.3421966666666663</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.12546955838841767</c:v>
+                  <c:v>0.1526851492773067</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2808,10 +2808,10 @@
                   <c:v>3.5680948493639999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.0244761776666667</c:v>
+                  <c:v>2.8862255499999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.53861867169733324</c:v>
+                  <c:v>0.67686929936400009</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2877,10 +2877,10 @@
                   <c:v>4.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.16010461155555558</c:v>
+                  <c:v>0.15278613333333332</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6348953884444439</c:v>
+                  <c:v>4.6422138666666664</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2946,10 +2946,10 @@
                   <c:v>0.89999999999999991</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.1926258607777778</c:v>
+                  <c:v>0.18382081666666664</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.70237413922222214</c:v>
+                  <c:v>0.7111791833333333</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3259,10 +3259,10 @@
                   <c:v>89.914599659044001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.6286777499999996</c:v>
+                  <c:v>5.3713874999999982</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>83.382041907905304</c:v>
+                  <c:v>83.440017977571969</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3328,10 +3328,10 @@
                   <c:v>4.2403446035919998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.5022883777777785</c:v>
+                  <c:v>3.3421966666666663</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.12546955838841767</c:v>
+                  <c:v>0.1526851492773067</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3397,10 +3397,10 @@
                   <c:v>3.5680948493639999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.0244761776666667</c:v>
+                  <c:v>2.8862255499999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.53861867169733324</c:v>
+                  <c:v>0.67686929936400009</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3466,10 +3466,10 @@
                   <c:v>4.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.16010461155555558</c:v>
+                  <c:v>0.15278613333333332</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6348953884444439</c:v>
+                  <c:v>4.6422138666666664</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3535,10 +3535,10 @@
                   <c:v>0.89999999999999991</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.1926258607777778</c:v>
+                  <c:v>0.18382081666666664</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.70237413922222214</c:v>
+                  <c:v>0.7111791833333333</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3832,10 +3832,10 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0" formatCode="0.00">
-                  <c:v>5.6286777499999996</c:v>
+                  <c:v>5.3713874999999982</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.1276970166666658</c:v>
+                  <c:v>3.9390174999999976</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3895,10 +3895,10 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0" formatCode="0.00">
-                  <c:v>3.5022883777777785</c:v>
+                  <c:v>3.3421966666666663</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.5022883777777785</c:v>
+                  <c:v>3.3421966666666663</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3958,10 +3958,10 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0" formatCode="0.00">
-                  <c:v>3.0244761776666667</c:v>
+                  <c:v>2.8862255499999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.0244761776666667</c:v>
+                  <c:v>2.8862255499999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4021,10 +4021,10 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0" formatCode="0.00">
-                  <c:v>0.16010461155555558</c:v>
+                  <c:v>0.15278613333333332</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.16010461155555558</c:v>
+                  <c:v>0.15278613333333332</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4084,10 +4084,10 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0" formatCode="0.00">
-                  <c:v>0.1926258607777778</c:v>
+                  <c:v>0.18382081666666664</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.1926258607777778</c:v>
+                  <c:v>0.18382081666666664</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9288,7 +9288,7 @@
       </c>
       <c r="B10" s="85"/>
       <c r="C10" s="183">
-        <v>42.402999999999999</v>
+        <v>40.58</v>
       </c>
       <c r="D10" s="85">
         <v>41.37</v>
@@ -9309,7 +9309,7 @@
       </c>
       <c r="B11" s="118"/>
       <c r="C11" s="184">
-        <v>35.680999999999997</v>
+        <v>34.049999999999997</v>
       </c>
       <c r="D11" s="118">
         <v>32.049999999999997</v>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="C15" s="35">
         <f>C13*C11</f>
-        <v>33.772066500000001</v>
+        <v>32.228324999999998</v>
       </c>
       <c r="D15" s="35">
         <f>D13*D11</f>
@@ -9404,7 +9404,7 @@
       </c>
       <c r="C16" s="127">
         <f>C6*1000/C15</f>
-        <v>7.994772839855683</v>
+        <v>8.377723632860226</v>
       </c>
       <c r="D16" s="127">
         <f>D6*1000/D15</f>
@@ -9432,7 +9432,7 @@
       </c>
       <c r="C17" s="35">
         <f>C5*1000/C16</f>
-        <v>35.022883777777778</v>
+        <v>33.421966666666663</v>
       </c>
       <c r="D17" s="35">
         <f>D5*1000/D16</f>
@@ -9460,7 +9460,7 @@
       </c>
       <c r="C18" s="129">
         <f>C17/C10</f>
-        <v>0.82595296978463273</v>
+        <v>0.82360686709380637</v>
       </c>
       <c r="D18" s="129">
         <f>D17/D10</f>
@@ -9488,7 +9488,7 @@
       </c>
       <c r="C19" s="132">
         <f>C17-C10</f>
-        <v>-7.3801162222222203</v>
+        <v>-7.1580333333333357</v>
       </c>
       <c r="D19" s="132">
         <f>D17-D10</f>
@@ -9516,7 +9516,7 @@
       </c>
       <c r="C20" s="134">
         <f>C19/C10</f>
-        <v>-0.17404703021536733</v>
+        <v>-0.1763931329061936</v>
       </c>
       <c r="D20" s="134">
         <f>D19/D10</f>
@@ -9544,7 +9544,7 @@
       </c>
       <c r="C21" s="13">
         <f>C10*C16</f>
-        <v>339.00235272840052</v>
+        <v>339.96802502146795</v>
       </c>
       <c r="D21" s="13">
         <f>D10*D16</f>
@@ -9572,7 +9572,7 @@
       </c>
       <c r="C22" s="11">
         <f>C11*C16</f>
-        <v>285.26148969889061</v>
+        <v>285.26148969889067</v>
       </c>
       <c r="D22" s="11">
         <f>D11*D16</f>
@@ -9931,7 +9931,7 @@
       </c>
       <c r="B11" s="5">
         <f>B15/B19*1000</f>
-        <v>85.624017114854396</v>
+        <v>89.725420107933019</v>
       </c>
       <c r="C11" s="49">
         <f>'Datos fabricación'!B6</f>
@@ -9946,7 +9946,7 @@
       </c>
       <c r="B12" s="35">
         <f>'Estándar técnico'!C10</f>
-        <v>42.402999999999999</v>
+        <v>40.58</v>
       </c>
       <c r="C12" s="35">
         <f>C14/C11*1000</f>
@@ -9959,7 +9959,7 @@
       </c>
       <c r="B13" s="35">
         <f>'Estándar técnico'!C11</f>
-        <v>35.680999999999997</v>
+        <v>34.049999999999997</v>
       </c>
       <c r="C13" s="35">
         <f>C15/C11*1000</f>
@@ -9973,7 +9973,7 @@
       </c>
       <c r="B14" s="35">
         <f>B$4/B$22*C$2</f>
-        <v>3.6307151977211705</v>
+        <v>3.6410575479799228</v>
       </c>
       <c r="C14" s="85">
         <f>'Datos fabricación'!B9</f>
@@ -10017,7 +10017,7 @@
       </c>
       <c r="B17" s="25">
         <f>B14/B15</f>
-        <v>1.1883915809534487</v>
+        <v>1.1917767988252572</v>
       </c>
       <c r="C17" s="25">
         <f>C14/C15</f>
@@ -10030,7 +10030,7 @@
       </c>
       <c r="B18" s="16">
         <f>B12</f>
-        <v>42.402999999999999</v>
+        <v>40.58</v>
       </c>
       <c r="C18" s="16">
         <f>C31*C2/C11</f>
@@ -10044,7 +10044,7 @@
       </c>
       <c r="B19" s="16">
         <f>B13</f>
-        <v>35.680999999999997</v>
+        <v>34.049999999999997</v>
       </c>
       <c r="C19" s="16">
         <f>C32*C2/C11</f>
@@ -10058,7 +10058,7 @@
       </c>
       <c r="B20" s="16">
         <f>B8/B21</f>
-        <v>35.022883777777771</v>
+        <v>33.42196666666667</v>
       </c>
       <c r="C20" s="16">
         <f>C8/C21</f>
@@ -10072,7 +10072,7 @@
       </c>
       <c r="B21" s="16">
         <f>(B5*1000/B19)/B23</f>
-        <v>7.9947728398556848</v>
+        <v>8.3777236328602243</v>
       </c>
       <c r="C21" s="16">
         <f>(C5*1000/C19)/C23</f>
@@ -10086,7 +10086,7 @@
       </c>
       <c r="B22" s="193">
         <f>'Estándar técnico'!C18</f>
-        <v>0.82595296978463273</v>
+        <v>0.82360686709380637</v>
       </c>
       <c r="C22" s="193">
         <f>(C4*C2)/C14</f>
@@ -10113,7 +10113,7 @@
       </c>
       <c r="B24" s="8">
         <f>B18-B20</f>
-        <v>7.3801162222222274</v>
+        <v>7.1580333333333286</v>
       </c>
       <c r="C24" s="8">
         <f>C18-C20</f>
@@ -10127,7 +10127,7 @@
       </c>
       <c r="B25" s="15">
         <f>B24/B18</f>
-        <v>0.17404703021536749</v>
+        <v>0.17639313290619341</v>
       </c>
       <c r="C25" s="15">
         <f>C24/C18</f>
@@ -10153,7 +10153,7 @@
       </c>
       <c r="B27" s="16">
         <f>B24-B26</f>
-        <v>7.3801162222222274</v>
+        <v>7.1580333333333286</v>
       </c>
       <c r="C27" s="16">
         <f>C24-C26</f>
@@ -10167,7 +10167,7 @@
       </c>
       <c r="B28" s="29">
         <f>B27/B18</f>
-        <v>0.17404703021536749</v>
+        <v>0.17639313290619341</v>
       </c>
       <c r="C28" s="29">
         <f>C27/C18</f>
@@ -10207,7 +10207,7 @@
       </c>
       <c r="B31" s="13">
         <f>B14/C2*1000</f>
-        <v>339.00235272840058</v>
+        <v>339.96802502146801</v>
       </c>
       <c r="C31" s="12">
         <f>C14/C2*1000</f>
@@ -10215,15 +10215,15 @@
       </c>
       <c r="D31" s="140">
         <f>(B31-C31)*C2/1000</f>
-        <v>-4.5979930719030511E-2</v>
+        <v>-3.5637580460278366E-2</v>
       </c>
       <c r="E31" s="140">
         <f>D31*B34</f>
-        <v>-0.25503775556248476</v>
+        <v>-0.19767164482709984</v>
       </c>
       <c r="F31" s="140">
         <f>E31/C2</f>
-        <v>-2.3813049072127425E-2</v>
+        <v>-1.8456736211680657E-2</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -10264,11 +10264,11 @@
       <c r="D33" s="52"/>
       <c r="E33" s="19">
         <f>SUM(E31:E32)</f>
-        <v>-1.3387188124138076</v>
+        <v>-1.2813527016784227</v>
       </c>
       <c r="F33" s="149">
         <f>SUM(F31:F32)</f>
-        <v>-0.12499708799381956</v>
+        <v>-0.1196407751333728</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -10376,7 +10376,7 @@
       </c>
       <c r="B39" s="19">
         <f>B14</f>
-        <v>3.6307151977211705</v>
+        <v>3.6410575479799228</v>
       </c>
       <c r="C39" s="19">
         <f>C14</f>
@@ -10384,15 +10384,15 @@
       </c>
       <c r="D39" s="19">
         <f>B39-C39</f>
-        <v>-4.5979930719030282E-2</v>
+        <v>-3.5637580460277984E-2</v>
       </c>
       <c r="E39" s="19">
         <f>D39*B34</f>
-        <v>-0.25503775556248348</v>
+        <v>-0.19767164482709773</v>
       </c>
       <c r="F39" s="140">
         <f>E39/C2</f>
-        <v>-2.3813049072127307E-2</v>
+        <v>-1.8456736211680459E-2</v>
       </c>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -10430,11 +10430,11 @@
       <c r="D41" s="52"/>
       <c r="E41" s="149">
         <f>SUM(E39:E40)</f>
-        <v>-1.3387188124138121</v>
+        <v>-1.2813527016784263</v>
       </c>
       <c r="F41" s="149">
         <f>SUM(F39:F40)</f>
-        <v>-0.12499708799381998</v>
+        <v>-0.11964077513337312</v>
       </c>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -10475,23 +10475,23 @@
       </c>
       <c r="B45" s="19">
         <f>B$4/B$22*C$2</f>
-        <v>3.6307151977211705</v>
+        <v>3.6410575479799228</v>
       </c>
       <c r="C45" s="19">
         <f>(C$4/B$22)*C$2</f>
-        <v>3.5788478377537247</v>
+        <v>3.5890424401516379</v>
       </c>
       <c r="D45" s="19">
         <f>B45-C45</f>
-        <v>5.1867359967445736E-2</v>
+        <v>5.201510782828489E-2</v>
       </c>
       <c r="E45" s="19">
         <f>D45*B$34</f>
-        <v>0.28769367126457795</v>
+        <v>0.2885131871322254</v>
       </c>
       <c r="F45" s="19">
         <f>E45/$C$2</f>
-        <v>2.6862154179699154E-2</v>
+        <v>2.6938672934848307E-2</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
       </c>
       <c r="B46" s="19">
         <f>B$4/B$22*C$2</f>
-        <v>3.6307151977211705</v>
+        <v>3.6410575479799228</v>
       </c>
       <c r="C46" s="145">
         <f>(B$4/C$22)*C$2</f>
@@ -10508,15 +10508,15 @@
       </c>
       <c r="D46" s="19">
         <f>B46-C46</f>
-        <v>-9.9265367363090995E-2</v>
+        <v>-8.8923017104338697E-2</v>
       </c>
       <c r="E46" s="19">
         <f>D46*B$34</f>
-        <v>-0.55059709967962411</v>
+        <v>-0.49323098894423834</v>
       </c>
       <c r="F46" s="19">
         <f t="shared" ref="F46:F57" si="0">E46/$C$2</f>
-        <v>-5.1409626487359854E-2</v>
+        <v>-4.6053313626913006E-2</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -10527,15 +10527,15 @@
       <c r="C47" s="19"/>
       <c r="D47" s="19">
         <f>(B22-C22)*(B4-C4)*C2</f>
-        <v>9.4166399755722121E-4</v>
+        <v>8.4115695828221998E-4</v>
       </c>
       <c r="E47" s="19">
         <f>D47*B$34</f>
-        <v>5.2231455914654454E-3</v>
+        <v>4.6656612865941987E-3</v>
       </c>
       <c r="F47" s="19">
         <f t="shared" si="0"/>
-        <v>4.8768866400237583E-4</v>
+        <v>4.3563597447191394E-4</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -10546,15 +10546,15 @@
       <c r="C48" s="146"/>
       <c r="D48" s="146">
         <f>SUM(D45:D47)</f>
-        <v>-4.6456343398088039E-2</v>
+        <v>-3.6066752317771587E-2</v>
       </c>
       <c r="E48" s="146">
         <f>SUM(E45:E47)</f>
-        <v>-0.25768028282358069</v>
+        <v>-0.20005214052541873</v>
       </c>
       <c r="F48" s="25">
         <f t="shared" si="0"/>
-        <v>-2.4059783643658326E-2</v>
+        <v>-1.8679004717592783E-2</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -10664,11 +10664,11 @@
       <c r="D54" s="159"/>
       <c r="E54" s="80">
         <f>E53+E48</f>
-        <v>-1.3674484785174221</v>
+        <v>-1.3098203362192602</v>
       </c>
       <c r="F54" s="80">
         <f>F53+F48</f>
-        <v>-0.12767959650022614</v>
+        <v>-0.12229881757416061</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -10680,11 +10680,11 @@
       <c r="D55" s="153"/>
       <c r="E55" s="140">
         <f>SUM(E45,E50)</f>
-        <v>1.8540446187499631</v>
+        <v>1.8548641346176105</v>
       </c>
       <c r="F55" s="19">
         <f t="shared" si="0"/>
-        <v>0.17311340978057543</v>
+        <v>0.1731899285357246</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -10693,11 +10693,11 @@
       </c>
       <c r="E56" s="19">
         <f>SUM(E46,E51)</f>
-        <v>-3.3455527292535061</v>
+        <v>-3.2881866185181199</v>
       </c>
       <c r="F56" s="19">
         <f t="shared" si="0"/>
-        <v>-0.31237653867913218</v>
+        <v>-0.30702022581868532</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -10707,11 +10707,11 @@
       <c r="D57" s="4"/>
       <c r="E57" s="19">
         <f>SUM(E47+E52)</f>
-        <v>0.1240596319861207</v>
+        <v>0.12350214768124945</v>
       </c>
       <c r="F57" s="25">
         <f t="shared" si="0"/>
-        <v>1.1583532398330596E-2</v>
+        <v>1.1531479708800134E-2</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -10723,7 +10723,7 @@
       <c r="D58" s="155"/>
       <c r="E58" s="156">
         <f>1-ABS(E57/E54)</f>
-        <v>0.90927655854308653</v>
+        <v>0.90571061979558731</v>
       </c>
       <c r="F58" s="156"/>
     </row>
@@ -10829,51 +10829,51 @@
       <c r="D5" s="69"/>
       <c r="E5" s="62">
         <f>B$21*(1-B22)</f>
-        <v>5.6286777499999996</v>
+        <v>5.3713874999999982</v>
       </c>
       <c r="F5" s="63">
         <f>E5/SUM($E$5:$E$9)</f>
-        <v>0.44999999999999996</v>
+        <v>0.45</v>
       </c>
       <c r="G5" s="62">
         <f>B5-E5</f>
-        <v>84.285921909044006</v>
+        <v>84.543212159044003</v>
       </c>
       <c r="H5" s="70">
         <f>G5/SUM($G$5:$G$9)</f>
-        <v>0.9270862435103977</v>
+        <v>0.92410463846298097</v>
       </c>
       <c r="I5" s="62">
         <f>I10-SUM(I6:I9)</f>
-        <v>0.90388000113870537</v>
+        <v>1.1031941814720403</v>
       </c>
       <c r="J5" s="86">
         <f>1-SUM(J6:J9)</f>
-        <v>0.59020546753782099</v>
+        <v>0.59195130850336564</v>
       </c>
       <c r="K5" s="62">
         <f>G5-I5</f>
-        <v>83.382041907905304</v>
+        <v>83.440017977571969</v>
       </c>
       <c r="L5" s="63">
         <f>K5/SUM($K$5:$K$9)</f>
-        <v>0.93285825130616251</v>
+        <v>0.93101157202522711</v>
       </c>
       <c r="M5" s="62">
         <f>K5*(1-H19)</f>
-        <v>0.25014612572371614</v>
+        <v>0.25032005393271611</v>
       </c>
       <c r="N5" s="63">
         <f>M5/SUM($M$5:$M$9)</f>
-        <v>4.0013751952533864E-2</v>
+        <v>3.8910250799775968E-2</v>
       </c>
       <c r="O5" s="64">
         <f>O10-SUM(O6:O9)</f>
-        <v>4.1276970166666658</v>
+        <v>3.9390174999999976</v>
       </c>
       <c r="P5" s="65">
         <f>O5/$O$10</f>
-        <v>0.37499999999999994</v>
+        <v>0.37499999999999989</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -10894,23 +10894,23 @@
       </c>
       <c r="E6" s="62">
         <f>B$21*B23</f>
-        <v>3.5022883777777785</v>
+        <v>3.3421966666666663</v>
       </c>
       <c r="F6" s="63">
         <f>E6/SUM($E$5:$E$9)</f>
-        <v>0.28000000000000003</v>
+        <v>0.28000000000000008</v>
       </c>
       <c r="G6" s="62">
         <f t="shared" ref="G6:G10" si="1">B6-E6</f>
-        <v>0.73805622581422137</v>
+        <v>0.89814793692533357</v>
       </c>
       <c r="H6" s="70">
         <f>G6/SUM($G$5:$G$9)</f>
-        <v>8.1181027435157961E-3</v>
+        <v>9.8172597579718329E-3</v>
       </c>
       <c r="I6" s="62">
         <f>G6*B33</f>
-        <v>0.6125866674258037</v>
+        <v>0.74546278764802687</v>
       </c>
       <c r="J6" s="63">
         <f>B32</f>
@@ -10918,23 +10918,23 @@
       </c>
       <c r="K6" s="62">
         <f t="shared" ref="K6:K10" si="2">G6-I6</f>
-        <v>0.12546955838841767</v>
+        <v>0.1526851492773067</v>
       </c>
       <c r="L6" s="63">
         <f>K6/SUM($K$5:$K$9)</f>
-        <v>1.4037232736474746E-3</v>
+        <v>1.703638665223934E-3</v>
       </c>
       <c r="M6" s="62">
         <f>K6</f>
-        <v>0.12546955838841767</v>
+        <v>0.1526851492773067</v>
       </c>
       <c r="N6" s="63">
         <f t="shared" ref="N6:N9" si="3">M6/SUM($M$5:$M$9)</f>
-        <v>2.0070299999342022E-2</v>
+        <v>2.373368556950747E-2</v>
       </c>
       <c r="O6" s="64">
         <f>E6</f>
-        <v>3.5022883777777785</v>
+        <v>3.3421966666666663</v>
       </c>
       <c r="P6" s="65">
         <f t="shared" ref="P6:P9" si="4">O6/$O$10</f>
@@ -10959,50 +10959,50 @@
       </c>
       <c r="E7" s="62">
         <f>(B21*B26)-SUM(E8:E9)</f>
-        <v>3.0244761776666667</v>
+        <v>2.8862255499999998</v>
       </c>
       <c r="F7" s="63">
         <f>E7/SUM($E$5:$E$9)</f>
-        <v>0.24179999999999999</v>
+        <v>0.24180000000000007</v>
       </c>
       <c r="G7" s="62">
         <f t="shared" si="1"/>
-        <v>0.54361867169733324</v>
+        <v>0.68186929936400009</v>
       </c>
       <c r="H7" s="70">
         <f>G7/SUM($G$5:$G$9)</f>
-        <v>5.9794255177022023E-3</v>
+        <v>7.4532131708266135E-3</v>
       </c>
       <c r="I7" s="97">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="J7" s="63">
         <f>I7/I10</f>
-        <v>3.2648441540596208E-3</v>
+        <v>2.682897165544778E-3</v>
       </c>
       <c r="K7" s="62">
         <f t="shared" si="2"/>
-        <v>0.53861867169733324</v>
+        <v>0.67686929936400009</v>
       </c>
       <c r="L7" s="63">
         <f>K7/SUM($K$5:$K$9)</f>
-        <v>6.0259362891997665E-3</v>
+        <v>7.5524090925516993E-3</v>
       </c>
       <c r="M7" s="62">
         <f>K7</f>
-        <v>0.53861867169733324</v>
+        <v>0.67686929936400009</v>
       </c>
       <c r="N7" s="63">
         <f t="shared" si="3"/>
-        <v>8.6158255955179175E-2</v>
+        <v>0.10521392027184959</v>
       </c>
       <c r="O7" s="64">
         <f t="shared" ref="O7:O9" si="6">E7</f>
-        <v>3.0244761776666667</v>
+        <v>2.8862255499999998</v>
       </c>
       <c r="P7" s="65">
         <f t="shared" si="4"/>
-        <v>0.27477272727272728</v>
+        <v>0.27477272727272734</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -11023,50 +11023,50 @@
       </c>
       <c r="E8" s="62">
         <f>B29*B21</f>
-        <v>0.16010461155555558</v>
+        <v>0.15278613333333332</v>
       </c>
       <c r="F8" s="63">
         <f>E8/SUM($E$5:$E$9)</f>
-        <v>1.2800000000000002E-2</v>
+        <v>1.2800000000000004E-2</v>
       </c>
       <c r="G8" s="62">
         <f t="shared" si="1"/>
-        <v>4.6398953884444438</v>
+        <v>4.6472138666666662</v>
       </c>
       <c r="H8" s="70">
         <f>G8/SUM($G$5:$G$9)</f>
-        <v>5.10356069972892E-2</v>
+        <v>5.079664919801307E-2</v>
       </c>
       <c r="I8" s="97">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="J8" s="63">
         <f>I8/I10</f>
-        <v>3.2648441540596208E-3</v>
+        <v>2.682897165544778E-3</v>
       </c>
       <c r="K8" s="62">
         <f t="shared" si="2"/>
-        <v>4.6348953884444439</v>
+        <v>4.6422138666666664</v>
       </c>
       <c r="L8" s="63">
         <f>K8/SUM($K$5:$K$9)</f>
-        <v>5.1854096015383842E-2</v>
+        <v>5.179714643451238E-2</v>
       </c>
       <c r="M8" s="62">
         <f>K8</f>
-        <v>4.6348953884444439</v>
+        <v>4.6422138666666664</v>
       </c>
       <c r="N8" s="63">
         <f t="shared" si="3"/>
-        <v>0.74140486430718211</v>
+        <v>0.72159502596923164</v>
       </c>
       <c r="O8" s="64">
         <f t="shared" si="6"/>
-        <v>0.16010461155555558</v>
+        <v>0.15278613333333332</v>
       </c>
       <c r="P8" s="65">
         <f t="shared" si="4"/>
-        <v>1.4545454545454547E-2</v>
+        <v>1.4545454545454549E-2</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -11087,46 +11087,46 @@
       </c>
       <c r="E9" s="62">
         <f>B30*B21</f>
-        <v>0.1926258607777778</v>
+        <v>0.18382081666666664</v>
       </c>
       <c r="F9" s="63">
         <f>E9/SUM($E$5:$E$9)</f>
-        <v>1.54E-2</v>
+        <v>1.5400000000000002E-2</v>
       </c>
       <c r="G9" s="62">
         <f t="shared" si="1"/>
-        <v>0.70737413922222214</v>
+        <v>0.7161791833333333</v>
       </c>
       <c r="H9" s="70">
         <f>G9/SUM($G$5:$G$9)</f>
-        <v>7.780621231095095E-3</v>
+        <v>7.8282394102075093E-3</v>
       </c>
       <c r="I9" s="97">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="J9" s="63">
         <f>I9/I10</f>
-        <v>3.2648441540596208E-3</v>
+        <v>2.682897165544778E-3</v>
       </c>
       <c r="K9" s="62">
         <f t="shared" si="2"/>
-        <v>0.70237413922222214</v>
+        <v>0.7111791833333333</v>
       </c>
       <c r="L9" s="63">
         <f>K9/SUM($K$5:$K$9)</f>
-        <v>7.8579931156062682E-3</v>
+        <v>7.9352337824849881E-3</v>
       </c>
       <c r="M9" s="62">
         <f>K9</f>
-        <v>0.70237413922222214</v>
+        <v>0.7111791833333333</v>
       </c>
       <c r="N9" s="63">
         <f t="shared" si="3"/>
-        <v>0.11235282778576293</v>
+        <v>0.11054711738963548</v>
       </c>
       <c r="O9" s="64">
         <f t="shared" si="6"/>
-        <v>0.1926258607777778</v>
+        <v>0.18382081666666664</v>
       </c>
       <c r="P9" s="65">
         <f t="shared" si="4"/>
@@ -11148,15 +11148,15 @@
       <c r="D10" s="91"/>
       <c r="E10" s="92">
         <f t="shared" si="7"/>
-        <v>12.508172777777778</v>
+        <v>11.936416666666663</v>
       </c>
       <c r="F10" s="93">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="G10" s="92">
         <f t="shared" si="1"/>
-        <v>90.914866334222239</v>
+        <v>91.486622445333353</v>
       </c>
       <c r="H10" s="94">
         <f t="shared" si="7"/>
@@ -11164,35 +11164,35 @@
       </c>
       <c r="I10" s="92">
         <f>I6/J6</f>
-        <v>1.5314666685645091</v>
+        <v>1.8636569691200671</v>
       </c>
       <c r="J10" s="94">
         <f t="shared" si="7"/>
-        <v>0.99999999999999978</v>
+        <v>1</v>
       </c>
       <c r="K10" s="92">
         <f t="shared" si="2"/>
-        <v>89.383399665657734</v>
+        <v>89.622965476213281</v>
       </c>
       <c r="L10" s="95">
         <f t="shared" si="7"/>
-        <v>0.99999999999999989</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="M10" s="92">
         <f>SUM(M5:M9)</f>
-        <v>6.2515038834761327</v>
+        <v>6.4332675525740219</v>
       </c>
       <c r="N10" s="95">
         <f>SUM(N5:N9)</f>
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="O10" s="96">
         <f>E10*(1-H20)</f>
-        <v>11.007192044444444</v>
+        <v>10.504046666666664</v>
       </c>
       <c r="P10" s="90">
         <f>SUM(P5:P9)</f>
-        <v>0.99999999999999989</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
@@ -11215,24 +11215,24 @@
       <c r="G12" s="26"/>
       <c r="H12" s="26">
         <f>1-H5</f>
-        <v>7.2913756489602299E-2</v>
+        <v>7.5895361537019035E-2</v>
       </c>
       <c r="I12" s="26"/>
       <c r="J12" s="26">
         <f>1-J5</f>
-        <v>0.40979453246217901</v>
+        <v>0.40804869149663436</v>
       </c>
       <c r="L12" s="26">
         <f>1-L5</f>
-        <v>6.7141748693837489E-2</v>
+        <v>6.8988427974772892E-2</v>
       </c>
       <c r="N12" s="26">
         <f>1-N5</f>
-        <v>0.95998624804746613</v>
+        <v>0.96108974920022405</v>
       </c>
       <c r="P12" s="26">
         <f>1-P5</f>
-        <v>0.625</v>
+        <v>0.62500000000000011</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -11246,24 +11246,24 @@
       <c r="G13" s="33"/>
       <c r="H13" s="33">
         <f>H6/H12</f>
-        <v>0.11133842411031805</v>
+        <v>0.12935256594282546</v>
       </c>
       <c r="I13" s="33"/>
       <c r="J13" s="33">
         <f>J6/J12</f>
-        <v>0.97609891863776166</v>
+        <v>0.98027516895811262</v>
       </c>
       <c r="L13" s="33">
         <f>L6/L12</f>
-        <v>2.0906861989078838E-2</v>
+        <v>2.4694556974785776E-2</v>
       </c>
       <c r="N13" s="33">
         <f>N6/N12</f>
-        <v>2.0906861989078884E-2</v>
+        <v>2.4694556974785738E-2</v>
       </c>
       <c r="P13" s="33">
         <f>P6/P12</f>
-        <v>0.50909090909090915</v>
+        <v>0.50909090909090904</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
@@ -11279,29 +11279,29 @@
       <c r="E14" s="57"/>
       <c r="F14" s="26">
         <f>SUM(F7:F9)</f>
-        <v>0.27</v>
+        <v>0.27000000000000007</v>
       </c>
       <c r="G14" s="26"/>
       <c r="H14" s="26">
         <f>SUM(H7:H9)</f>
-        <v>6.4795653746086493E-2</v>
+        <v>6.6078101779047188E-2</v>
       </c>
       <c r="I14" s="26"/>
       <c r="J14" s="26">
         <f>SUM(J7:J9)</f>
-        <v>9.7945324621788628E-3</v>
+        <v>8.0486914966343345E-3</v>
       </c>
       <c r="L14" s="26">
         <f>SUM(L7:L9)</f>
-        <v>6.5738025420189874E-2</v>
+        <v>6.7284789309549065E-2</v>
       </c>
       <c r="N14" s="26">
         <f>SUM(N7:N9)</f>
-        <v>0.93991594804812417</v>
+        <v>0.93735606363071677</v>
       </c>
       <c r="P14" s="26">
         <f>SUM(P7:P9)</f>
-        <v>0.30681818181818182</v>
+        <v>0.30681818181818188</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
@@ -11315,24 +11315,24 @@
       <c r="G15" s="26"/>
       <c r="H15" s="26">
         <f>H5/(1-H6)</f>
-        <v>0.93467402326294147</v>
+        <v>0.93326676067601844</v>
       </c>
       <c r="I15" s="26"/>
       <c r="J15" s="26">
         <f>J5/(1-J6)</f>
-        <v>0.98367577922970173</v>
+        <v>0.98658551417227613</v>
       </c>
       <c r="L15" s="26">
         <f>L5/(1-L6)</f>
-        <v>0.93416956686870933</v>
+        <v>0.93260038610219353</v>
       </c>
       <c r="N15" s="26">
         <f>N5/(1-N6)</f>
-        <v>4.0833288298647338E-2</v>
+        <v>3.9856184961656049E-2</v>
       </c>
       <c r="P15" s="26">
         <f>P5/(1-P6)</f>
-        <v>0.54999999999999993</v>
+        <v>0.54999999999999982</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -11352,7 +11352,7 @@
       </c>
       <c r="H18" s="33">
         <f>G10/B10</f>
-        <v>0.87905815875095017</v>
+        <v>0.88458648315545685</v>
       </c>
       <c r="I18" s="33"/>
       <c r="J18" s="33"/>
@@ -11378,7 +11378,7 @@
       </c>
       <c r="B20" s="59">
         <f>'Estándar técnico'!C16</f>
-        <v>7.994772839855683</v>
+        <v>8.377723632860226</v>
       </c>
       <c r="E20" t="s">
         <v>87</v>
@@ -11393,7 +11393,7 @@
       </c>
       <c r="B21" s="28">
         <f>B18/B20</f>
-        <v>12.508172777777778</v>
+        <v>11.936416666666664</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="F22" s="33">
         <f>SUM(E7:E9)/B7</f>
-        <v>0.94650136629691195</v>
+        <v>0.90323621878338178</v>
       </c>
       <c r="G22" s="33"/>
       <c r="H22" s="28">
@@ -11432,7 +11432,7 @@
       </c>
       <c r="F23" s="33">
         <f>E6/B6</f>
-        <v>0.82594428170082845</v>
+        <v>0.78818987113346595</v>
       </c>
       <c r="G23" s="33"/>
       <c r="H23" s="28">
@@ -11455,7 +11455,7 @@
       </c>
       <c r="F24" s="59">
         <f>B18/E10</f>
-        <v>7.994772839855683</v>
+        <v>8.3777236328602278</v>
       </c>
       <c r="G24" s="59"/>
       <c r="H24" s="59"/>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="F26" s="56">
         <f>SUM(E7:E9)</f>
-        <v>3.3772066500000002</v>
+        <v>3.2228324999999995</v>
       </c>
       <c r="G26" s="56"/>
       <c r="H26" s="56"/>
@@ -11497,7 +11497,7 @@
       </c>
       <c r="F27" s="56">
         <f>E6</f>
-        <v>3.5022883777777785</v>
+        <v>3.3421966666666663</v>
       </c>
       <c r="G27" s="56"/>
       <c r="H27" s="56"/>
@@ -11510,7 +11510,7 @@
       </c>
       <c r="F28" s="56">
         <f>SUM(F26:F27)</f>
-        <v>6.8794950277777787</v>
+        <v>6.5650291666666654</v>
       </c>
       <c r="G28" s="56"/>
       <c r="H28" s="56"/>
@@ -11542,7 +11542,7 @@
       </c>
       <c r="F30" s="28">
         <f>F28/F29</f>
-        <v>12.508172777777778</v>
+        <v>11.936416666666663</v>
       </c>
       <c r="G30" s="28"/>
       <c r="H30" s="28"/>

</xml_diff>